<commit_message>
Update BOC USD rates (auto)
</commit_message>
<xml_diff>
--- a/data/2026/2026-01.xlsx
+++ b/data/2026/2026-01.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Daily Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Published Values'!$A$1:$J$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Published Values'!$A$1:$J$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Daily Summary'!$A$1:$E$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1848,8 +1848,60 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-01-04 17:19:01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>697.87</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>697.87</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>700.81</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>700.81</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>702.88</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026/01/04 17:19:01</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-01-04 09:31:16</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://www.bankofchina.com/sourcedb/whpj/enindex_1619.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J27"/>
+  <autoFilter ref="A1:J28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1950,7 +2002,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" t="n">
         <v>702.88</v>

</xml_diff>